<commit_message>
Updated software versions and vcf processing for phylogenetic analysis
</commit_message>
<xml_diff>
--- a/data/Complete_coffee_genotype_list.xlsx
+++ b/data/Complete_coffee_genotype_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://griffitheduau.sharepoint.com/sites/Fordlab308/Shared Documents/General/Projects/Fawad_coffee/SNP_Calling_Coffee/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="13_ncr:1_{27C57BC3-2D71-1142-ADF3-12440635F372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3C2E593-EF6A-4C96-945C-3A12AF1C63A0}"/>
+  <xr:revisionPtr revIDLastSave="93" documentId="13_ncr:1_{27C57BC3-2D71-1142-ADF3-12440635F372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6FAC42E-50E2-40F8-87CA-3869B86549AC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29DE232E-A8DD-024C-8432-AAD26E21EE26}"/>
+    <workbookView xWindow="4350" yWindow="2325" windowWidth="21600" windowHeight="11385" xr2:uid="{29DE232E-A8DD-024C-8432-AAD26E21EE26}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="37">
   <si>
     <t>Mundo Novo</t>
   </si>
@@ -111,18 +111,9 @@
     <t>Fawad Grafting Project Australia</t>
   </si>
   <si>
-    <t>Arabica</t>
-  </si>
-  <si>
-    <t>Robusta</t>
-  </si>
-  <si>
     <t>Allotetraploid</t>
   </si>
   <si>
-    <t>Liberica spp</t>
-  </si>
-  <si>
     <t>Diploid</t>
   </si>
   <si>
@@ -147,9 +138,6 @@
     <t>Sequencing_ID</t>
   </si>
   <si>
-    <t>Genotype code in numbers</t>
-  </si>
-  <si>
     <t>Species</t>
   </si>
   <si>
@@ -165,10 +153,19 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>Low Quality DNA (did not pass QC)</t>
-  </si>
-  <si>
     <t>Low quality DNA (did not pass QC)</t>
+  </si>
+  <si>
+    <t>Genotype_code</t>
+  </si>
+  <si>
+    <t>C. robusta</t>
+  </si>
+  <si>
+    <t>C. arabica</t>
+  </si>
+  <si>
+    <t>C. liberica spp</t>
   </si>
 </sst>
 </file>
@@ -275,6 +272,30 @@
   </cellStyles>
   <dxfs count="16">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -292,30 +313,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -571,7 +568,7 @@
     <tableColumn id="1" xr3:uid="{E757C568-5541-43B4-B69A-8CFF5665A297}" name="Sequencing_ID" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{0258FEC7-7616-4299-B638-E4BF3CF9B9B4}" name="Genotype" dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{90859089-3808-4F98-801A-A99A6904DA27}" name="Replicate" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{A96737C0-F08F-40EF-82A6-CBC3B3A9D2CB}" name="Genotype code in numbers" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{A96737C0-F08F-40EF-82A6-CBC3B3A9D2CB}" name="Genotype_code" dataDxfId="10"/>
     <tableColumn id="5" xr3:uid="{3B744408-B239-4A4C-8E72-FF73F682ACD9}" name="Species" dataDxfId="9"/>
     <tableColumn id="6" xr3:uid="{5E4BC0FD-2E7C-4188-A681-85AB0BAD1AEA}" name="Ploidy_level" dataDxfId="8"/>
     <tableColumn id="7" xr3:uid="{33AF2362-64C3-42A5-B3F5-0BF4EF7A6570}" name="Chromosome_number" dataDxfId="7"/>
@@ -584,7 +581,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3CE996A6-5421-41A5-8298-DF7C9F04585C}" name="Table2" displayName="Table2" ref="A1:A20" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="2" tableBorderDxfId="3" totalsRowBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3CE996A6-5421-41A5-8298-DF7C9F04585C}" name="Table2" displayName="Table2" ref="A1:A20" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1" totalsRowBorderDxfId="0">
   <autoFilter ref="A1:A20" xr:uid="{3CE996A6-5421-41A5-8298-DF7C9F04585C}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{1710035C-A738-441F-A06E-43416A5ABB60}" name="Genotype"/>
@@ -918,49 +915,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51B98EA8-8A8F-3041-B974-E03C027512EC}">
-  <dimension ref="A1:P59"/>
-  <sheetFormatPr defaultColWidth="31.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J59"/>
+  <sheetFormatPr defaultColWidth="31.25" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="31.19921875" style="1"/>
-    <col min="3" max="3" width="35.69921875" style="1" customWidth="1"/>
-    <col min="4" max="7" width="31.19921875" style="1"/>
-    <col min="8" max="8" width="35.69921875" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="31.19921875" style="1"/>
+    <col min="1" max="1" width="17.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="31.25" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -974,10 +977,10 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G2" s="1">
         <v>22</v>
@@ -990,7 +993,7 @@
       </c>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1004,10 +1007,10 @@
         <v>1</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G3" s="1">
         <v>22</v>
@@ -1020,7 +1023,7 @@
       </c>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1034,10 +1037,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G4" s="1">
         <v>22</v>
@@ -1050,7 +1053,7 @@
       </c>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1064,10 +1067,10 @@
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G5" s="1">
         <v>22</v>
@@ -1080,7 +1083,7 @@
       </c>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1094,10 +1097,10 @@
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G6" s="1">
         <v>22</v>
@@ -1110,7 +1113,7 @@
       </c>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1124,10 +1127,10 @@
         <v>2</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G7" s="1">
         <v>22</v>
@@ -1140,7 +1143,7 @@
       </c>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1154,10 +1157,10 @@
         <v>3</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G8" s="1">
         <v>44</v>
@@ -1170,7 +1173,7 @@
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1184,10 +1187,10 @@
         <v>3</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G9" s="1">
         <v>44</v>
@@ -1200,7 +1203,7 @@
       </c>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1214,10 +1217,10 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G10" s="1">
         <v>44</v>
@@ -1230,7 +1233,7 @@
       </c>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1244,10 +1247,10 @@
         <v>4</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G11" s="1">
         <v>44</v>
@@ -1260,7 +1263,7 @@
       </c>
       <c r="J11" s="3"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1274,10 +1277,10 @@
         <v>4</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G12" s="1">
         <v>44</v>
@@ -1290,7 +1293,7 @@
       </c>
       <c r="J12" s="3"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1304,10 +1307,10 @@
         <v>4</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G13" s="1">
         <v>44</v>
@@ -1320,7 +1323,7 @@
       </c>
       <c r="J13" s="3"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1334,10 +1337,10 @@
         <v>5</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G14" s="1">
         <v>44</v>
@@ -1350,7 +1353,7 @@
       </c>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1364,10 +1367,10 @@
         <v>5</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G15" s="1">
         <v>44</v>
@@ -1380,7 +1383,7 @@
       </c>
       <c r="J15" s="3"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1394,10 +1397,10 @@
         <v>5</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G16" s="1">
         <v>44</v>
@@ -1410,7 +1413,7 @@
       </c>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1424,10 +1427,10 @@
         <v>6</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G17" s="1">
         <v>44</v>
@@ -1440,7 +1443,7 @@
       </c>
       <c r="J17" s="3"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1454,10 +1457,10 @@
         <v>6</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G18" s="1">
         <v>44</v>
@@ -1470,7 +1473,7 @@
       </c>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1484,10 +1487,10 @@
         <v>6</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G19" s="1">
         <v>44</v>
@@ -1500,7 +1503,7 @@
       </c>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1514,10 +1517,10 @@
         <v>7</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G20" s="1">
         <v>44</v>
@@ -1530,7 +1533,7 @@
       </c>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1544,10 +1547,10 @@
         <v>7</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G21" s="1">
         <v>44</v>
@@ -1560,7 +1563,7 @@
       </c>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1574,10 +1577,10 @@
         <v>7</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G22" s="1">
         <v>44</v>
@@ -1590,12 +1593,12 @@
       </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C23" s="1">
         <v>1</v>
@@ -1604,10 +1607,10 @@
         <v>8</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G23" s="1">
         <v>44</v>
@@ -1620,12 +1623,12 @@
       </c>
       <c r="J23" s="3"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C24" s="1">
         <v>2</v>
@@ -1634,10 +1637,10 @@
         <v>8</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G24" s="1">
         <v>44</v>
@@ -1650,12 +1653,12 @@
       </c>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C25" s="1">
         <v>3</v>
@@ -1664,10 +1667,10 @@
         <v>8</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G25" s="1">
         <v>44</v>
@@ -1680,7 +1683,7 @@
       </c>
       <c r="J25" s="3"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1694,10 +1697,10 @@
         <v>9</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G26" s="1">
         <v>22</v>
@@ -1710,7 +1713,7 @@
       </c>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1724,10 +1727,10 @@
         <v>9</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G27" s="1">
         <v>22</v>
@@ -1740,7 +1743,7 @@
       </c>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1754,10 +1757,10 @@
         <v>9</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G28" s="1">
         <v>22</v>
@@ -1770,12 +1773,12 @@
       </c>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C29" s="1">
         <v>1</v>
@@ -1784,10 +1787,10 @@
         <v>10</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G29" s="1">
         <v>44</v>
@@ -1800,12 +1803,12 @@
       </c>
       <c r="J29" s="3"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C30" s="1">
         <v>2</v>
@@ -1814,10 +1817,10 @@
         <v>10</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G30" s="1">
         <v>44</v>
@@ -1830,12 +1833,12 @@
       </c>
       <c r="J30" s="3"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C31" s="1">
         <v>3</v>
@@ -1844,10 +1847,10 @@
         <v>10</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G31" s="1">
         <v>44</v>
@@ -1860,7 +1863,7 @@
       </c>
       <c r="J31" s="3"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1874,10 +1877,10 @@
         <v>11</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G32" s="1">
         <v>44</v>
@@ -1890,7 +1893,7 @@
       </c>
       <c r="J32" s="3"/>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1904,10 +1907,10 @@
         <v>11</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G33" s="1">
         <v>44</v>
@@ -1920,7 +1923,7 @@
       </c>
       <c r="J33" s="3"/>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1934,10 +1937,10 @@
         <v>11</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G34" s="1">
         <v>44</v>
@@ -1950,7 +1953,7 @@
       </c>
       <c r="J34" s="3"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1964,10 +1967,10 @@
         <v>12</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G35" s="1">
         <v>44</v>
@@ -1980,7 +1983,7 @@
       </c>
       <c r="J35" s="3"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1994,10 +1997,10 @@
         <v>12</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G36" s="1">
         <v>44</v>
@@ -2010,7 +2013,7 @@
       </c>
       <c r="J36" s="3"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -2024,10 +2027,10 @@
         <v>12</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G37" s="1">
         <v>44</v>
@@ -2040,7 +2043,7 @@
       </c>
       <c r="J37" s="3"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -2054,10 +2057,10 @@
         <v>13</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G38" s="1">
         <v>44</v>
@@ -2070,7 +2073,7 @@
       </c>
       <c r="J38" s="3"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -2084,10 +2087,10 @@
         <v>13</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G39" s="1">
         <v>44</v>
@@ -2100,7 +2103,7 @@
       </c>
       <c r="J39" s="3"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -2114,10 +2117,10 @@
         <v>13</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G40" s="1">
         <v>44</v>
@@ -2130,7 +2133,7 @@
       </c>
       <c r="J40" s="3"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -2144,10 +2147,10 @@
         <v>14</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G41" s="1">
         <v>44</v>
@@ -2160,7 +2163,7 @@
       </c>
       <c r="J41" s="3"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -2174,10 +2177,10 @@
         <v>14</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G42" s="1">
         <v>44</v>
@@ -2190,7 +2193,7 @@
       </c>
       <c r="J42" s="3"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -2204,10 +2207,10 @@
         <v>14</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G43" s="1">
         <v>44</v>
@@ -2220,7 +2223,7 @@
       </c>
       <c r="J43" s="3"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -2234,10 +2237,10 @@
         <v>15</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G44" s="1">
         <v>44</v>
@@ -2250,7 +2253,7 @@
       </c>
       <c r="J44" s="3"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -2264,10 +2267,10 @@
         <v>15</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G45" s="1">
         <v>44</v>
@@ -2280,7 +2283,7 @@
       </c>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -2294,10 +2297,10 @@
         <v>15</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G46" s="1">
         <v>44</v>
@@ -2309,13 +2312,10 @@
         <v>17</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P46" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -2329,10 +2329,10 @@
         <v>16</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G47" s="1">
         <v>44</v>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="J47" s="3"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -2359,10 +2359,10 @@
         <v>16</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G48" s="1">
         <v>44</v>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -2389,10 +2389,10 @@
         <v>16</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G49" s="1">
         <v>44</v>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="J49" s="3"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -2419,10 +2419,10 @@
         <v>17</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G50" s="1">
         <v>44</v>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="J50" s="3"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -2449,10 +2449,10 @@
         <v>17</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G51" s="1">
         <v>44</v>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="J51" s="3"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -2479,10 +2479,10 @@
         <v>17</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G52" s="1">
         <v>44</v>
@@ -2495,12 +2495,12 @@
       </c>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C53" s="1">
         <v>1</v>
@@ -2516,12 +2516,12 @@
       </c>
       <c r="J53" s="3"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C54" s="1">
         <v>2</v>
@@ -2537,12 +2537,12 @@
       </c>
       <c r="J54" s="3"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C55" s="1">
         <v>3</v>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="J55" s="3"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -2572,10 +2572,10 @@
         <v>1</v>
       </c>
       <c r="E56" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="G56" s="1">
         <v>22</v>
@@ -2588,12 +2588,12 @@
       </c>
       <c r="J56" s="3"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C57" s="3">
         <v>1</v>
@@ -2601,11 +2601,11 @@
       <c r="D57" s="3">
         <v>10</v>
       </c>
-      <c r="E57" s="3" t="s">
-        <v>18</v>
+      <c r="E57" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G57" s="3">
         <v>44</v>
@@ -2618,12 +2618,12 @@
       </c>
       <c r="J57" s="3"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C58" s="3">
         <v>2</v>
@@ -2631,11 +2631,11 @@
       <c r="D58" s="3">
         <v>10</v>
       </c>
-      <c r="E58" s="3" t="s">
-        <v>18</v>
+      <c r="E58" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G58" s="3">
         <v>44</v>
@@ -2648,12 +2648,12 @@
       </c>
       <c r="J58" s="3"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C59" s="3">
         <v>3</v>
@@ -2661,11 +2661,11 @@
       <c r="D59" s="3">
         <v>10</v>
       </c>
-      <c r="E59" s="3" t="s">
-        <v>18</v>
+      <c r="E59" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G59" s="3">
         <v>44</v>
@@ -2690,109 +2690,109 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA56E02D-FFB2-41CA-AEA5-A83AD98372DB}">
   <dimension ref="A1:A20"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.796875" customWidth="1"/>
+    <col min="1" max="1" width="10.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -3044,7 +3044,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{618C0BF5-15DE-4B8A-98CD-C558B8C2BAF4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{618C0BF5-15DE-4B8A-98CD-C558B8C2BAF4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b546f376-916d-4a96-a17a-18f0544e88ec"/>
+    <ds:schemaRef ds:uri="c4d6b203-dae6-48f7-b66f-8d2f96fb6de7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>